<commit_message>
- persistance save completion
</commit_message>
<xml_diff>
--- a/Documents/MMO_Project_Design_Data_Tracker.xlsx
+++ b/Documents/MMO_Project_Design_Data_Tracker.xlsx
@@ -1326,7 +1326,7 @@
       </c>
       <c r="B4" s="33" t="inlineStr">
         <is>
-          <t>Extend persistence to Inventory, Equipment/Ammo, and window layout (v2 save scope)</t>
+          <t>Additional mob variety (more content beyond Poring/Poporing)</t>
         </is>
       </c>
       <c r="C4" s="33" t="inlineStr">
@@ -1341,7 +1341,7 @@
       </c>
       <c r="B5" s="33" t="inlineStr">
         <is>
-          <t>Additional mob variety (more content beyond Poring/Poporing)</t>
+          <t>Hook the Mage's selected element into damage (selection already exists; needs a resistance/multiplier step)</t>
         </is>
       </c>
       <c r="C5" s="33" t="inlineStr">
@@ -1356,7 +1356,7 @@
       </c>
       <c r="B6" s="33" t="inlineStr">
         <is>
-          <t>Hook the Mage's selected element into damage (selection already exists; needs a resistance/multiplier step)</t>
+          <t>Author icons for FireBolt, Mammonite, Envenom (Sprite Editor — the skill data/wiring itself is done)</t>
         </is>
       </c>
       <c r="C6" s="33" t="inlineStr">
@@ -1371,12 +1371,12 @@
       </c>
       <c r="B7" s="33" t="inlineStr">
         <is>
-          <t>Author icons for FireBolt, Mammonite, Envenom (Sprite Editor — the skill data/wiring itself is done)</t>
+          <t>Skill buffs / debuffs (temporary stat modifiers)</t>
         </is>
       </c>
       <c r="C7" s="33" t="inlineStr">
         <is>
-          <t>Near-term</t>
+          <t>Mid-term</t>
         </is>
       </c>
     </row>
@@ -1386,7 +1386,7 @@
       </c>
       <c r="B8" s="33" t="inlineStr">
         <is>
-          <t>Skill buffs / debuffs (temporary stat modifiers)</t>
+          <t>Ground-targeted AoE skills (no fixed target)</t>
         </is>
       </c>
       <c r="C8" s="33" t="inlineStr">
@@ -1401,7 +1401,7 @@
       </c>
       <c r="B9" s="33" t="inlineStr">
         <is>
-          <t>Ground-targeted AoE skills (no fixed target)</t>
+          <t>Full elemental damage and enemy resistances</t>
         </is>
       </c>
       <c r="C9" s="33" t="inlineStr">
@@ -1416,7 +1416,7 @@
       </c>
       <c r="B10" s="33" t="inlineStr">
         <is>
-          <t>Full elemental damage and enemy resistances</t>
+          <t>Quest system</t>
         </is>
       </c>
       <c r="C10" s="33" t="inlineStr">
@@ -1431,7 +1431,7 @@
       </c>
       <c r="B11" s="33" t="inlineStr">
         <is>
-          <t>Quest system</t>
+          <t>Shops / economy (Zeny), including an ammo restock source</t>
         </is>
       </c>
       <c r="C11" s="33" t="inlineStr">
@@ -1446,7 +1446,7 @@
       </c>
       <c r="B12" s="33" t="inlineStr">
         <is>
-          <t>Shops / economy (Zeny), including an ammo restock source</t>
+          <t>Class evolution / promotion</t>
         </is>
       </c>
       <c r="C12" s="33" t="inlineStr">
@@ -1461,12 +1461,12 @@
       </c>
       <c r="B13" s="33" t="inlineStr">
         <is>
-          <t>Class evolution / promotion</t>
+          <t>Authoritative multiplayer server</t>
         </is>
       </c>
       <c r="C13" s="33" t="inlineStr">
         <is>
-          <t>Mid-term</t>
+          <t>Long-term</t>
         </is>
       </c>
     </row>
@@ -1476,7 +1476,7 @@
       </c>
       <c r="B14" s="33" t="inlineStr">
         <is>
-          <t>Authoritative multiplayer server</t>
+          <t>Revisit grid-based (SQM) movement</t>
         </is>
       </c>
       <c r="C14" s="33" t="inlineStr">
@@ -1486,19 +1486,9 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="18" t="n">
-        <v>12</v>
-      </c>
-      <c r="B15" s="18" t="inlineStr">
-        <is>
-          <t>Revisit grid-based (SQM) movement</t>
-        </is>
-      </c>
-      <c r="C15" s="18" t="inlineStr">
-        <is>
-          <t>Long-term</t>
-        </is>
-      </c>
+      <c r="A15" s="18" t="n"/>
+      <c r="B15" s="18" t="n"/>
+      <c r="C15" s="18" t="n"/>
     </row>
   </sheetData>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
@@ -2528,7 +2518,7 @@
       </c>
       <c r="D56" s="33" t="inlineStr">
         <is>
-          <t>v1: JSON file save via Project.Persistence (ISaveParticipant/ISaveRepository), auto-loads on Start and auto-saves on quit. Covers Base/Job level+experience, the six base stats and unspent points, class, Zeny, learned skills+levels (via new SkillDatabase asset), hotbar assignments, and the Mage's selected element.</t>
+          <t>v1+v2: JSON file save via Project.Persistence (ISaveParticipant/ISaveRepository). PlayerSaveController discovers every ISaveParticipant in the loaded scene (not just the Player's own components), auto-loads on Start, auto-saves on quit. Covers Base/Job level+experience, the six base stats and unspent points, class, Zeny, learned skills+levels, hotbar assignments, the Mage's selected element, full inventory contents, equipped items (incl. the Ammo stack), and window layout/open/minimized state.</t>
         </is>
       </c>
     </row>
@@ -2543,14 +2533,14 @@
           <t>Persistence coverage: Inventory, Equipment/Ammo, window layout (v2)</t>
         </is>
       </c>
-      <c r="C57" s="35" t="inlineStr">
-        <is>
-          <t>Planned</t>
+      <c r="C57" s="34" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="D57" s="33" t="inlineStr">
         <is>
-          <t>Not yet part of the save system; still lost when Play Mode stops</t>
+          <t>Inventory (via new ItemDatabase asset resolving items to stable ids, mirroring SkillDatabase), equipped items and ammo count (via EquipmentManager), and every WindowPanel's open/minimized state and position now implement ISaveParticipant.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
- Project.World assembly: MapTransitionService, WarpPortal, MapSpawnPoint, PersistentPlayerAnchor, PersistAcrossScenes, MapBootstrap - Prototype_Map02 scene, linked to Prototype_Map01 via warp portals - Camera target and respawn point wiring - Player HP/MP bar billboard camera fix - Warp disc + destination label per portal
</commit_message>
<xml_diff>
--- a/Documents/MMO_Project_Design_Data_Tracker.xlsx
+++ b/Documents/MMO_Project_Design_Data_Tracker.xlsx
@@ -570,7 +570,7 @@
     <row r="3" ht="15" customHeight="1" s="19">
       <c r="A3" s="21" t="inlineStr">
         <is>
-          <t>Last updated: July 23, 2026</t>
+          <t>Last updated: August 31, 2026</t>
         </is>
       </c>
     </row>
@@ -1326,7 +1326,7 @@
       </c>
       <c r="B4" s="33" t="inlineStr">
         <is>
-          <t>Additional mob variety (more content beyond Poring/Poporing)</t>
+          <t>Save / persistence system</t>
         </is>
       </c>
       <c r="C4" s="33" t="inlineStr">
@@ -1341,7 +1341,7 @@
       </c>
       <c r="B5" s="33" t="inlineStr">
         <is>
-          <t>Hook the Mage's selected element into damage (selection already exists; needs a resistance/multiplier step)</t>
+          <t>Additional mob variety (more content beyond Poring/Poporing)</t>
         </is>
       </c>
       <c r="C5" s="33" t="inlineStr">
@@ -1356,7 +1356,7 @@
       </c>
       <c r="B6" s="33" t="inlineStr">
         <is>
-          <t>Author icons for FireBolt, Mammonite, Envenom (Sprite Editor — the skill data/wiring itself is done)</t>
+          <t>Hook the Mage's selected element into damage (selection already exists; needs a resistance/multiplier step)</t>
         </is>
       </c>
       <c r="C6" s="33" t="inlineStr">
@@ -1371,12 +1371,12 @@
       </c>
       <c r="B7" s="33" t="inlineStr">
         <is>
-          <t>Skill buffs / debuffs (temporary stat modifiers)</t>
+          <t>Author icons for FireBolt, Mammonite, Envenom (Sprite Editor — the skill data/wiring itself is done)</t>
         </is>
       </c>
       <c r="C7" s="33" t="inlineStr">
         <is>
-          <t>Mid-term</t>
+          <t>Near-term</t>
         </is>
       </c>
     </row>
@@ -1386,7 +1386,7 @@
       </c>
       <c r="B8" s="33" t="inlineStr">
         <is>
-          <t>Ground-targeted AoE skills (no fixed target)</t>
+          <t>Skill buffs / debuffs (temporary stat modifiers)</t>
         </is>
       </c>
       <c r="C8" s="33" t="inlineStr">
@@ -1401,7 +1401,7 @@
       </c>
       <c r="B9" s="33" t="inlineStr">
         <is>
-          <t>Full elemental damage and enemy resistances</t>
+          <t>Ground-targeted AoE skills (no fixed target)</t>
         </is>
       </c>
       <c r="C9" s="33" t="inlineStr">
@@ -1416,7 +1416,7 @@
       </c>
       <c r="B10" s="33" t="inlineStr">
         <is>
-          <t>Quest system</t>
+          <t>Full elemental damage and enemy resistances</t>
         </is>
       </c>
       <c r="C10" s="33" t="inlineStr">
@@ -1431,7 +1431,7 @@
       </c>
       <c r="B11" s="33" t="inlineStr">
         <is>
-          <t>Shops / economy (Zeny), including an ammo restock source</t>
+          <t>Quest system</t>
         </is>
       </c>
       <c r="C11" s="33" t="inlineStr">
@@ -1446,7 +1446,7 @@
       </c>
       <c r="B12" s="33" t="inlineStr">
         <is>
-          <t>Class evolution / promotion</t>
+          <t>Shops / economy (Zeny), including an ammo restock source</t>
         </is>
       </c>
       <c r="C12" s="33" t="inlineStr">
@@ -1461,12 +1461,12 @@
       </c>
       <c r="B13" s="33" t="inlineStr">
         <is>
-          <t>Authoritative multiplayer server</t>
+          <t>Class evolution / promotion</t>
         </is>
       </c>
       <c r="C13" s="33" t="inlineStr">
         <is>
-          <t>Long-term</t>
+          <t>Mid-term</t>
         </is>
       </c>
     </row>
@@ -1476,19 +1476,29 @@
       </c>
       <c r="B14" s="33" t="inlineStr">
         <is>
+          <t>Authoritative multiplayer server</t>
+        </is>
+      </c>
+      <c r="C14" s="33" t="inlineStr">
+        <is>
+          <t>Long-term</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="18" t="n">
+        <v>12</v>
+      </c>
+      <c r="B15" s="18" t="inlineStr">
+        <is>
           <t>Revisit grid-based (SQM) movement</t>
         </is>
       </c>
-      <c r="C14" s="33" t="inlineStr">
+      <c r="C15" s="18" t="inlineStr">
         <is>
           <t>Long-term</t>
         </is>
       </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="18" t="n"/>
-      <c r="B15" s="18" t="n"/>
-      <c r="C15" s="18" t="n"/>
     </row>
   </sheetData>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
@@ -2472,7 +2482,7 @@
       </c>
       <c r="B54" s="33" t="inlineStr">
         <is>
-          <t>Assembly Definitions (13 assemblies)</t>
+          <t>Assembly Definitions (12 assemblies)</t>
         </is>
       </c>
       <c r="C54" s="34" t="inlineStr">
@@ -2511,14 +2521,14 @@
           <t>Save / persistence system</t>
         </is>
       </c>
-      <c r="C56" s="34" t="inlineStr">
-        <is>
-          <t>Done</t>
+      <c r="C56" s="35" t="inlineStr">
+        <is>
+          <t>Planned</t>
         </is>
       </c>
       <c r="D56" s="33" t="inlineStr">
         <is>
-          <t>v1+v2: JSON file save via Project.Persistence (ISaveParticipant/ISaveRepository). PlayerSaveController discovers every ISaveParticipant in the loaded scene (not just the Player's own components), auto-loads on Start, auto-saves on quit. Covers Base/Job level+experience, the six base stats and unspent points, class, Zeny, learned skills+levels, hotbar assignments, the Mage's selected element, full inventory contents, equipped items (incl. the Ammo stack), and window layout/open/minimized state.</t>
+          <t>Largest known gap</t>
         </is>
       </c>
     </row>
@@ -2530,17 +2540,17 @@
       </c>
       <c r="B57" s="33" t="inlineStr">
         <is>
-          <t>Persistence coverage: Inventory, Equipment/Ammo, window layout (v2)</t>
-        </is>
-      </c>
-      <c r="C57" s="34" t="inlineStr">
-        <is>
-          <t>Done</t>
+          <t>Authoritative server / multiplayer</t>
+        </is>
+      </c>
+      <c r="C57" s="35" t="inlineStr">
+        <is>
+          <t>Planned</t>
         </is>
       </c>
       <c r="D57" s="33" t="inlineStr">
         <is>
-          <t>Inventory (via new ItemDatabase asset resolving items to stable ids, mirroring SkillDatabase), equipped items and ammo count (via EquipmentManager), and every WindowPanel's open/minimized state and position now implement ISaveParticipant.</t>
+          <t>Fish-Networking under consideration</t>
         </is>
       </c>
     </row>
@@ -2552,7 +2562,7 @@
       </c>
       <c r="B58" s="33" t="inlineStr">
         <is>
-          <t>Authoritative server / multiplayer</t>
+          <t>Automated tests</t>
         </is>
       </c>
       <c r="C58" s="35" t="inlineStr">
@@ -2560,29 +2570,29 @@
           <t>Planned</t>
         </is>
       </c>
-      <c r="D58" s="33" t="inlineStr">
-        <is>
-          <t>Fish-Networking under consideration</t>
-        </is>
-      </c>
+      <c r="D58" s="33" t="n"/>
     </row>
     <row r="59" ht="23.85" customHeight="1" s="19">
       <c r="A59" s="33" t="inlineStr">
         <is>
-          <t>Technical</t>
+          <t>Content</t>
         </is>
       </c>
       <c r="B59" s="33" t="inlineStr">
         <is>
-          <t>Automated tests</t>
-        </is>
-      </c>
-      <c r="C59" s="35" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
-      <c r="D59" s="33" t="n"/>
+          <t>Mob variety</t>
+        </is>
+      </c>
+      <c r="C59" s="36" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="D59" s="33" t="inlineStr">
+        <is>
+          <t>Aggressive/Passive behavior modes done; only Poring/Poporing exist as content</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="33" t="inlineStr">
@@ -2592,29 +2602,25 @@
       </c>
       <c r="B60" s="33" t="inlineStr">
         <is>
-          <t>Mob variety</t>
-        </is>
-      </c>
-      <c r="C60" s="36" t="inlineStr">
-        <is>
-          <t>Partial</t>
-        </is>
-      </c>
-      <c r="D60" s="33" t="inlineStr">
-        <is>
-          <t>Aggressive/Passive behavior modes done; only Poring/Poporing exist as content</t>
-        </is>
-      </c>
+          <t>Quest system</t>
+        </is>
+      </c>
+      <c r="C60" s="35" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="D60" s="33" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="33" t="inlineStr">
         <is>
-          <t>Content</t>
+          <t>Character Stats</t>
         </is>
       </c>
       <c r="B61" s="33" t="inlineStr">
         <is>
-          <t>Quest system</t>
+          <t>Quasi-stats (Attack Range, Cast Time, Perfect Dodge, etc.)</t>
         </is>
       </c>
       <c r="C61" s="35" t="inlineStr">
@@ -2622,7 +2628,11 @@
           <t>Planned</t>
         </is>
       </c>
-      <c r="D61" s="33" t="n"/>
+      <c r="D61" s="33" t="inlineStr">
+        <is>
+          <t>Attack Range now implemented per-weapon for basic attacks (see GDD 3.6/4.1); remaining quasi-stats still planned — see Quasi-Stats sheet</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="33" t="inlineStr">
@@ -2632,17 +2642,17 @@
       </c>
       <c r="B62" s="33" t="inlineStr">
         <is>
-          <t>Quasi-stats (Attack Range, Cast Time, Perfect Dodge, etc.)</t>
-        </is>
-      </c>
-      <c r="C62" s="35" t="inlineStr">
-        <is>
-          <t>Planned</t>
+          <t>Attack Range (per-weapon, basic attacks)</t>
+        </is>
+      </c>
+      <c r="C62" s="34" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="D62" s="33" t="inlineStr">
         <is>
-          <t>Attack Range now implemented per-weapon for basic attacks (see GDD 3.6/4.1); remaining quasi-stats still planned — see Quasi-Stats sheet</t>
+          <t>See GDD 3.6 / 4.1; skill range remains separately defined per skill</t>
         </is>
       </c>
     </row>
@@ -2654,17 +2664,17 @@
       </c>
       <c r="B63" s="33" t="inlineStr">
         <is>
-          <t>Attack Range (per-weapon, basic attacks)</t>
-        </is>
-      </c>
-      <c r="C63" s="34" t="inlineStr">
-        <is>
-          <t>Done</t>
+          <t>Block Rate as a named sub-stat (currently a fixed Swordman-only chance)</t>
+        </is>
+      </c>
+      <c r="C63" s="35" t="inlineStr">
+        <is>
+          <t>Planned</t>
         </is>
       </c>
       <c r="D63" s="33" t="inlineStr">
         <is>
-          <t>See GDD 3.6 / 4.1; skill range remains separately defined per skill</t>
+          <t>Swordman block exists via IDamageModifier but is not yet a STR/VIT/shield-driven sub-stat</t>
         </is>
       </c>
     </row>
@@ -2676,7 +2686,7 @@
       </c>
       <c r="B64" s="33" t="inlineStr">
         <is>
-          <t>Block Rate as a named sub-stat (currently a fixed Swordman-only chance)</t>
+          <t>Stat Points Reset</t>
         </is>
       </c>
       <c r="C64" s="35" t="inlineStr">
@@ -2686,7 +2696,7 @@
       </c>
       <c r="D64" s="33" t="inlineStr">
         <is>
-          <t>Swordman block exists via IDamageModifier but is not yet a STR/VIT/shield-driven sub-stat</t>
+          <t>No reset mechanism exists yet</t>
         </is>
       </c>
     </row>
@@ -2698,39 +2708,39 @@
       </c>
       <c r="B65" s="33" t="inlineStr">
         <is>
-          <t>Stat Points Reset</t>
-        </is>
-      </c>
-      <c r="C65" s="35" t="inlineStr">
-        <is>
-          <t>Planned</t>
+          <t>Talent Stats (POW/STA/WIS/SPL/CON/CRT) and Lv.200+ substats</t>
+        </is>
+      </c>
+      <c r="C65" s="37" t="inlineStr">
+        <is>
+          <t>Out of scope</t>
         </is>
       </c>
       <c r="D65" s="33" t="inlineStr">
         <is>
-          <t>No reset mechanism exists yet</t>
+          <t>Assumes 4th-job content far beyond current roadmap</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="33" t="inlineStr">
         <is>
-          <t>Character Stats</t>
+          <t>World</t>
         </is>
       </c>
       <c r="B66" s="33" t="inlineStr">
         <is>
-          <t>Talent Stats (POW/STA/WIS/SPL/CON/CRT) and Lv.200+ substats</t>
+          <t>Multi-map navigation (separate scenes linked by warp portals)</t>
         </is>
       </c>
       <c r="C66" s="37" t="inlineStr">
         <is>
-          <t>Out of scope</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="D66" s="33" t="inlineStr">
         <is>
-          <t>Assumes 4th-job content far beyond current roadmap</t>
+          <t>Prototype_Map01 &lt;-&gt; Prototype_Map02 via WarpPortal + MapTransitionService; player/UI persist across scene loads (DontDestroyOnLoad). New maps still need their NavMesh baked manually in the Editor before they are walkable.</t>
         </is>
       </c>
     </row>

</xml_diff>